<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-10-12.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-10-12.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-10-12.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -521,10 +521,102 @@
       <c r="A11" t="str">
         <v>35</v>
       </c>
+      <c r="C11" t="str">
+        <v>211_海洋之心_Nautica_Rosa rugosa Thunb._20stems</v>
+      </c>
+      <c r="F11" t="str">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" t="str">
+        <v>160_卡布奇诺_Cappuccino_Rosa rugosa Thunb._20stems</v>
+      </c>
+      <c r="F12" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" t="str">
+        <v>284_可爱瓷_undefined_Rosa rugosa Thunb._20stems</v>
+      </c>
+      <c r="F13" t="str">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" t="str">
+        <v>279_完美甜蜜_undefined_Rosa rugosa Thunb._10stems</v>
+      </c>
+      <c r="F14" t="str">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>36</v>
+      </c>
+      <c r="C15" t="str">
+        <v>203_佛罗伊德_Floyd_Rosa rugosa Thunb._20stems</v>
+      </c>
+      <c r="F15" t="str">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" t="str">
+        <v>279_完美甜蜜_undefined_Rosa rugosa Thunb._10stems</v>
+      </c>
+      <c r="F16" t="str">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>37</v>
+      </c>
+      <c r="C17" t="str">
+        <v>195_闺蜜_Alter Ego_Rosa rugosa Thunb._20stems</v>
+      </c>
+      <c r="F17" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" t="str">
+        <v>279_完美甜蜜_undefined_Rosa rugosa Thunb._10stems</v>
+      </c>
+      <c r="F18" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="str">
+        <v>152_白荔枝_White Ohara_Rosa rugosa Thunb._20stems</v>
+      </c>
+      <c r="F19" t="str">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>38</v>
+      </c>
+      <c r="C20" t="str">
+        <v>594_绿毛球_undefined_undefined_1bunch</v>
+      </c>
+      <c r="F20" t="str">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>39</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -579,7 +671,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0202020161420309200</v>
+        <v>02020201614203092020514103610252410400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>